<commit_message>
panele(R-PANEL-SYNC): generatory eksportuja koszty surowcowe (jednostki Surowiec+ilosc, budynki koszt_surowce) + regen Panel-B/C
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fs7eokPtaxbQL7KGTXXeWS
</commit_message>
<xml_diff>
--- a/panele-sterowania/Panel-B.xlsx
+++ b/panele-sterowania/Panel-B.xlsx
@@ -4401,7 +4401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V37"/>
+  <dimension ref="A1:AA37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -4515,6 +4515,31 @@
           <t>techUnlock</t>
         </is>
       </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>koszt_surowce.drewno</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>koszt_surowce.kamien</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>koszt_surowce.cegla</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>koszt_surowce.braz</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>koszt_surowce.zelazo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4589,6 +4614,9 @@
           <t>Obróbka drewna</t>
         </is>
       </c>
+      <c r="W2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4663,6 +4691,12 @@
           <t>Murarstwo</t>
         </is>
       </c>
+      <c r="W3" t="n">
+        <v>3</v>
+      </c>
+      <c r="X3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4737,6 +4771,12 @@
           <t>Brązownictwo</t>
         </is>
       </c>
+      <c r="W4" t="n">
+        <v>4</v>
+      </c>
+      <c r="X4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4811,6 +4851,12 @@
           <t>Brązownictwo</t>
         </is>
       </c>
+      <c r="X5" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4885,6 +4931,12 @@
           <t>Hutnictwo żelaza</t>
         </is>
       </c>
+      <c r="Y6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4959,6 +5011,9 @@
           <t>Wymiana</t>
         </is>
       </c>
+      <c r="W7" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5033,6 +5088,9 @@
           <t>Żegluga</t>
         </is>
       </c>
+      <c r="W8" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5107,6 +5165,12 @@
           <t>Inżynieria</t>
         </is>
       </c>
+      <c r="Y9" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5181,6 +5245,9 @@
           <t>Handel</t>
         </is>
       </c>
+      <c r="Y10" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5255,6 +5322,12 @@
           <t>Garncarstwo</t>
         </is>
       </c>
+      <c r="W11" t="n">
+        <v>5</v>
+      </c>
+      <c r="X11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5329,6 +5402,9 @@
           <t>Warzelnia soli</t>
         </is>
       </c>
+      <c r="Y12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5403,6 +5479,12 @@
           <t>Garncarstwo</t>
         </is>
       </c>
+      <c r="W13" t="n">
+        <v>4</v>
+      </c>
+      <c r="X13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5477,6 +5559,12 @@
           <t>Garncarstwo</t>
         </is>
       </c>
+      <c r="W14" t="n">
+        <v>4</v>
+      </c>
+      <c r="X14" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5551,6 +5639,9 @@
           <t>Mistycyzm</t>
         </is>
       </c>
+      <c r="X15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5625,6 +5716,9 @@
           <t>Religia</t>
         </is>
       </c>
+      <c r="Y16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5699,6 +5793,9 @@
           <t>Pismo</t>
         </is>
       </c>
+      <c r="Y17" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5773,6 +5870,9 @@
           <t>Gospodarka wodna</t>
         </is>
       </c>
+      <c r="X18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5847,6 +5947,9 @@
           <t>Budownictwo</t>
         </is>
       </c>
+      <c r="Y19" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5921,6 +6024,12 @@
           <t>Waluta</t>
         </is>
       </c>
+      <c r="X20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5995,6 +6104,9 @@
           <t>Budownictwo</t>
         </is>
       </c>
+      <c r="Y21" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6069,6 +6181,15 @@
           <t>Wojskowość</t>
         </is>
       </c>
+      <c r="W22" t="n">
+        <v>6</v>
+      </c>
+      <c r="X22" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6143,6 +6264,12 @@
           <t>Handel</t>
         </is>
       </c>
+      <c r="W23" t="n">
+        <v>8</v>
+      </c>
+      <c r="X23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6217,6 +6344,9 @@
           <t>Murarstwo</t>
         </is>
       </c>
+      <c r="X24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6291,6 +6421,12 @@
           <t>-</t>
         </is>
       </c>
+      <c r="W25" t="n">
+        <v>8</v>
+      </c>
+      <c r="X25" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6365,6 +6501,12 @@
           <t>Hutnictwo żelaza</t>
         </is>
       </c>
+      <c r="Y26" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6513,6 +6655,12 @@
           <t>Inżynieria</t>
         </is>
       </c>
+      <c r="Y28" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6587,6 +6735,12 @@
           <t>Oblężnictwo</t>
         </is>
       </c>
+      <c r="Y29" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6661,6 +6815,9 @@
           <t>Filozofia</t>
         </is>
       </c>
+      <c r="Y30" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6735,6 +6892,9 @@
           <t>Filozofia</t>
         </is>
       </c>
+      <c r="Y31" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6809,6 +6969,9 @@
           <t>Prawo</t>
         </is>
       </c>
+      <c r="Y32" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6883,6 +7046,9 @@
           <t>Prawo</t>
         </is>
       </c>
+      <c r="Y33" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6957,6 +7123,9 @@
           <t>Kodeks</t>
         </is>
       </c>
+      <c r="Y34" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7031,6 +7200,9 @@
           <t>Medycyna</t>
         </is>
       </c>
+      <c r="Y35" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7178,6 +7350,12 @@
         <is>
           <t>Sztuka wojenna</t>
         </is>
+      </c>
+      <c r="Y37" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>